<commit_message>
assign 9mm muzzle loudness
for some reason excel decided to clear out a bunch of redundant zeros and added some more to some of the new stuff
</commit_message>
<xml_diff>
--- a/changes/9mm-muzzles.xlsx
+++ b/changes/9mm-muzzles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F62C69D5-1538-4BE1-8320-A841BC309B65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F4441C-33C5-4041-AB30-EE0BB3E1314C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="m4-barrels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>new</t>
   </si>
@@ -89,12 +89,6 @@
     <t>FD917</t>
   </si>
   <si>
-    <t>mp5_noveske_style_muzzle_brake_th</t>
-  </si>
-  <si>
-    <t>MP5 Noveske Style Muzzle Brake</t>
-  </si>
-  <si>
     <t>alphadog_alpha9_flipped</t>
   </si>
   <si>
@@ -104,123 +98,36 @@
     <t>alphadog_alpha9</t>
   </si>
   <si>
-    <t>Alpha Dog Alpha 9 9x19 Suppressor</t>
-  </si>
-  <si>
-    <t>vityaz_suppressor</t>
-  </si>
-  <si>
-    <t>Vityaz 9x19</t>
-  </si>
-  <si>
     <t>sig_srd9_9x19</t>
   </si>
   <si>
-    <t>Sig SRD 9 9x19mm</t>
-  </si>
-  <si>
     <t>9x19_naughty_9</t>
   </si>
   <si>
     <t>Naughty-9</t>
   </si>
   <si>
-    <t>wilson_combat_9x19_thread_protector</t>
-  </si>
-  <si>
-    <t>Wilson Combat 9x19</t>
-  </si>
-  <si>
     <t>9x19_thread_protector</t>
   </si>
   <si>
     <t>9x19 Thread Protector</t>
   </si>
   <si>
-    <t>silencerco_osprey9_gen1_9x19_suppressor</t>
-  </si>
-  <si>
-    <t>SilencerCo Osprey 9 Gen 1 9x19 Suppressor</t>
-  </si>
-  <si>
-    <t>silencerco_osprey9_gen1_9x19_suppressor_flipped</t>
-  </si>
-  <si>
-    <t>SilencerCo Osprey 9 Gen 1 9x19 Suppressor Flipped</t>
-  </si>
-  <si>
-    <t>vltor_vc9_9x19_compensator</t>
-  </si>
-  <si>
-    <t>VLTOR VC9 9x19 Compensator</t>
-  </si>
-  <si>
     <t>ips_9x19_1inch_barrel_extension</t>
   </si>
   <si>
-    <t>IPS 9x19 1in Barrel Extension</t>
-  </si>
-  <si>
     <t>wasatch_arms_comp_weight_compensator_10mm</t>
   </si>
   <si>
     <t>Wasatch Arms Comp Weight 10mm Compensator for Glock 20</t>
   </si>
   <si>
-    <t>rugged_suppressors_obsidian_9_9x19_piston</t>
-  </si>
-  <si>
-    <t>Rugged Suppressors Obsidian9 9x19 Piston</t>
-  </si>
-  <si>
-    <t>rugged_suppressors_obsidian_9_3lug_piston</t>
-  </si>
-  <si>
-    <t>Rugged Suppressors Obsidian9 3-Lug Piston</t>
-  </si>
-  <si>
-    <t>rugged_suppressors_obsidian_9_body</t>
-  </si>
-  <si>
-    <t>Rugged Suppressors Obsidian9 9x19 Body</t>
-  </si>
-  <si>
-    <t>rugged_suppressors_obsidian_9_extension</t>
-  </si>
-  <si>
-    <t>Rugged Suppressors Obsidian9 9x19 Extension</t>
-  </si>
-  <si>
-    <t>rugged_suppressors_obsidian_9_cap</t>
-  </si>
-  <si>
-    <t>Rugged Suppressors Obsidian9 9x19 Cap</t>
-  </si>
-  <si>
-    <t>radian_weapons_glock17_afterburner_micro_compensator</t>
-  </si>
-  <si>
     <t>Radian Weapons Glock 17 Gen5 AFTERBURNER Micro Compensator</t>
   </si>
   <si>
-    <t>irl weight</t>
-  </si>
-  <si>
-    <t>weight formula</t>
-  </si>
-  <si>
-    <t>izhmash_pp-19-01_vityaz_std_muzzle_brake_compensator</t>
-  </si>
-  <si>
-    <t>Izhmash PP-19-01 Vityaz Std.</t>
-  </si>
-  <si>
     <t>hk_mp5sd_9x19_suppressor</t>
   </si>
   <si>
-    <t>HK MP5SD 9x19 Suppressor</t>
-  </si>
-  <si>
     <t>9x19_rotor43_8chamber_pf940_suppressor</t>
   </si>
   <si>
@@ -228,6 +135,96 @@
   </si>
   <si>
     <t>barrel_deviation</t>
+  </si>
+  <si>
+    <t>muzzle_loudness</t>
+  </si>
+  <si>
+    <t>MPi54SD 9x19</t>
+  </si>
+  <si>
+    <t>mp5_nowa_style_muzzle_brake_th</t>
+  </si>
+  <si>
+    <t>MPi-54 Nowa Style</t>
+  </si>
+  <si>
+    <t>Alpha Dog Alpha 9 9x19</t>
+  </si>
+  <si>
+    <t>suppressors_inc_osprey9_gen1_9x19_suppressor</t>
+  </si>
+  <si>
+    <t>Suppressors Inc. Osprey 9 Gen 1 9x19</t>
+  </si>
+  <si>
+    <t>suppressors_inc_osprey9_gen1_9x19_suppressor_flipped</t>
+  </si>
+  <si>
+    <t>Suppressors Inc. Osprey 9 Gen 1 9x19 Flipped</t>
+  </si>
+  <si>
+    <t>resiliant_suppressors_obsidian_9_9x19_piston</t>
+  </si>
+  <si>
+    <t>Resiliant Suppressors Obsidian9 9x19 Piston</t>
+  </si>
+  <si>
+    <t>resiliant_suppressors_obsidian_9_3lug_piston</t>
+  </si>
+  <si>
+    <t>Resiliant Suppressors Obsidian9 3-Lug Piston</t>
+  </si>
+  <si>
+    <t>resiliant_suppressors_obsidian_9_body</t>
+  </si>
+  <si>
+    <t>Resiliant Suppressors Obsidian9 9x19 Body</t>
+  </si>
+  <si>
+    <t>resiliant_suppressors_obsidian_9_extension</t>
+  </si>
+  <si>
+    <t>Resiliant Suppressors Obsidian9 9x19 Extension</t>
+  </si>
+  <si>
+    <t>resiliant_suppressors_obsidian_9_cap</t>
+  </si>
+  <si>
+    <t>Resiliant Suppressors Obsidian9 9x19 Cap</t>
+  </si>
+  <si>
+    <t>ardian_weapons_glock17_afterburner_micro_compensator</t>
+  </si>
+  <si>
+    <t>IPS 1" 9x19</t>
+  </si>
+  <si>
+    <t>whitner_defense_9x19_thread_protector</t>
+  </si>
+  <si>
+    <t>Whitner Defense 9x19</t>
+  </si>
+  <si>
+    <t>vyctor_vc9_9x19_compensator</t>
+  </si>
+  <si>
+    <t>VYCTOR VC-9 9x19</t>
+  </si>
+  <si>
+    <t>SIC SRD 9 9x19mm</t>
+  </si>
+  <si>
+    <t>kazarov_pp-19-01_vityaz_std_muzzle_brake_compensator</t>
+  </si>
+  <si>
+    <t>Kazarov PP-19-01 Vityaz Std.</t>
+  </si>
+  <si>
+    <t>kazarov_pp-19-01_vityaz_9x19_suppressor</t>
+  </si>
+  <si>
+    <t>Kazarov PP-19-01 Vityaz 9x19</t>
   </si>
 </sst>
 </file>
@@ -1068,19 +1065,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="2" width="40.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1103,7 +1100,7 @@
         <v>8</v>
       </c>
       <c r="H2" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="I2" t="s">
         <v>9</v>
@@ -1118,24 +1115,21 @@
         <v>12</v>
       </c>
       <c r="M2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" t="s">
         <v>13</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>3</v>
       </c>
-      <c r="P2" t="s">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
         <v>56</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" t="s">
-        <v>31</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -1158,20 +1152,20 @@
       <c r="J3">
         <v>0</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>100</v>
       </c>
-      <c r="N3">
-        <f>C3-D3*20-E3*0.8-F3*0.6-H3*5+I3*15+J3/300</f>
+      <c r="O3">
+        <f>C3-D3*20-E3*0.8-F3*0.6-H3*10+I3*15+J3/200-M3*5</f>
         <v>2.8</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -1194,20 +1188,20 @@
       <c r="J4">
         <v>0</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>100</v>
       </c>
-      <c r="N4">
-        <f t="shared" ref="N4:N25" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*5+I4*15+J4/300</f>
+      <c r="O4">
+        <f t="shared" ref="O4:O28" si="0">C4-D4*20-E4*0.8-F4*0.6-H4*10+I4*15+J4/200-M4*5</f>
         <v>2.8</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C5">
         <v>-1</v>
@@ -1230,15 +1224,15 @@
       <c r="J5">
         <v>30</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>500</v>
       </c>
-      <c r="N5">
-        <f t="shared" si="0"/>
-        <v>-3.0500000000000003</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O5">
+        <f t="shared" si="0"/>
+        <v>-3.3000000000000007</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1266,20 +1260,20 @@
       <c r="J6">
         <v>10</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>500</v>
       </c>
-      <c r="N6">
-        <f t="shared" si="0"/>
-        <v>5.833333333333333</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O6">
+        <f t="shared" si="0"/>
+        <v>5.85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C7">
         <v>-1</v>
@@ -1303,19 +1297,22 @@
         <v>20</v>
       </c>
       <c r="M7">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="N7">
         <v>600</v>
       </c>
-      <c r="N7">
-        <f t="shared" si="0"/>
-        <v>7.8666666666666663</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O7">
+        <f t="shared" si="0"/>
+        <v>7.55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="C8">
         <v>-2</v>
@@ -1339,19 +1336,22 @@
         <v>20</v>
       </c>
       <c r="M8">
+        <v>0.04</v>
+      </c>
+      <c r="N8">
         <v>1800</v>
       </c>
-      <c r="N8">
-        <f t="shared" si="0"/>
-        <v>8.0666666666666664</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O8">
+        <f t="shared" si="0"/>
+        <v>7.8999999999999995</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C9">
         <v>-1</v>
@@ -1375,19 +1375,22 @@
         <v>0</v>
       </c>
       <c r="M9">
+        <v>0.03</v>
+      </c>
+      <c r="N9">
         <v>100</v>
       </c>
-      <c r="N9">
-        <f t="shared" si="0"/>
-        <v>7.2000000000000011</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O9">
+        <f t="shared" si="0"/>
+        <v>7.0500000000000007</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1411,19 +1414,22 @@
         <v>20</v>
       </c>
       <c r="M10">
+        <v>0.04</v>
+      </c>
+      <c r="N10">
         <v>1000</v>
       </c>
-      <c r="N10">
-        <f t="shared" si="0"/>
-        <v>6.2666666666666666</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O10">
+        <f t="shared" si="0"/>
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>-3</v>
@@ -1447,19 +1453,22 @@
         <v>-100</v>
       </c>
       <c r="M11">
+        <v>0.04</v>
+      </c>
+      <c r="N11">
         <v>1000</v>
       </c>
-      <c r="N11">
-        <f t="shared" si="0"/>
-        <v>2.6666666666666665</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O11">
+        <f t="shared" si="0"/>
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C12">
         <v>-2</v>
@@ -1483,19 +1492,22 @@
         <v>50</v>
       </c>
       <c r="M12">
+        <v>-0.05</v>
+      </c>
+      <c r="N12">
         <v>900</v>
       </c>
-      <c r="N12">
-        <f t="shared" si="0"/>
-        <v>6.916666666666667</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O12">
+        <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-M12*5</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="C13">
         <v>-4</v>
@@ -1519,19 +1531,22 @@
         <v>90</v>
       </c>
       <c r="M13">
+        <v>-0.15</v>
+      </c>
+      <c r="N13">
         <v>1500</v>
       </c>
-      <c r="N13">
-        <f t="shared" si="0"/>
-        <v>7.3999999999999977</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O13">
+        <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
+        <v>8.7999999999999972</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14">
         <v>-7</v>
@@ -1555,19 +1570,22 @@
         <v>150</v>
       </c>
       <c r="M14">
+        <v>-0.13</v>
+      </c>
+      <c r="N14">
         <v>1000</v>
       </c>
-      <c r="N14">
-        <f t="shared" si="0"/>
-        <v>2.9499999999999997</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O14">
+        <f t="shared" si="0"/>
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C15">
         <v>-8</v>
@@ -1591,19 +1609,22 @@
         <v>150</v>
       </c>
       <c r="M15">
+        <v>-0.13</v>
+      </c>
+      <c r="N15">
         <v>1000</v>
       </c>
-      <c r="N15">
-        <f t="shared" si="0"/>
-        <v>1.9499999999999997</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="O15">
+        <f t="shared" si="0"/>
+        <v>3.5999999999999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="C16">
         <v>-5</v>
@@ -1618,7 +1639,7 @@
         <v>-10</v>
       </c>
       <c r="H16">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="I16">
         <v>0.13</v>
@@ -1627,19 +1648,22 @@
         <v>150</v>
       </c>
       <c r="M16">
+        <v>-0.2</v>
+      </c>
+      <c r="N16">
         <v>1200</v>
       </c>
-      <c r="N16">
-        <f t="shared" si="0"/>
-        <v>7.3499999999999988</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O16">
+        <f t="shared" si="0"/>
+        <v>10.099999999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>-5</v>
@@ -1663,19 +1687,22 @@
         <v>100</v>
       </c>
       <c r="M17">
+        <v>-0.18</v>
+      </c>
+      <c r="N17">
         <v>1000</v>
       </c>
-      <c r="N17">
-        <f t="shared" si="0"/>
-        <v>7.0333333333333323</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O17">
+        <f t="shared" si="0"/>
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>-6</v>
@@ -1699,19 +1726,22 @@
         <v>150</v>
       </c>
       <c r="M18">
+        <v>-0.1</v>
+      </c>
+      <c r="N18">
         <v>1500</v>
       </c>
-      <c r="N18">
-        <f t="shared" si="0"/>
-        <v>7.2999999999999989</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O18">
+        <f t="shared" si="0"/>
+        <v>8.7999999999999989</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C19">
         <v>-6</v>
@@ -1735,14 +1765,17 @@
         <v>150</v>
       </c>
       <c r="M19">
+        <v>-0.1</v>
+      </c>
+      <c r="N19">
         <v>1500</v>
       </c>
-      <c r="N19">
-        <f t="shared" si="0"/>
-        <v>7.2999999999999989</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O19">
+        <f t="shared" si="0"/>
+        <v>8.7999999999999989</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1770,20 +1803,20 @@
       <c r="J20">
         <v>200</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>2000</v>
       </c>
-      <c r="N20">
-        <f t="shared" si="0"/>
-        <v>3.7166666666666677</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O20">
+        <f t="shared" si="0"/>
+        <v>4.8000000000000007</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
         <v>44</v>
-      </c>
-      <c r="B21" t="s">
-        <v>45</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1806,20 +1839,20 @@
       <c r="J21">
         <v>0</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>300</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <f t="shared" si="0"/>
         <v>-0.6</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B22" t="s">
         <v>46</v>
-      </c>
-      <c r="B22" t="s">
-        <v>47</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -1842,26 +1875,26 @@
       <c r="J22">
         <v>0</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>300</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <f t="shared" si="0"/>
         <v>-0.6</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
         <v>48</v>
-      </c>
-      <c r="B24" t="s">
-        <v>49</v>
       </c>
       <c r="C24">
         <v>-4</v>
@@ -1885,19 +1918,22 @@
         <v>70</v>
       </c>
       <c r="M24">
+        <v>-0.08</v>
+      </c>
+      <c r="N24">
         <v>1500</v>
       </c>
-      <c r="N24">
-        <f t="shared" si="0"/>
-        <v>8.1833333333333336</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O24">
+        <f t="shared" si="0"/>
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
         <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>51</v>
       </c>
       <c r="C25">
         <v>-3</v>
@@ -1921,19 +1957,22 @@
         <v>50</v>
       </c>
       <c r="M25">
+        <v>-0.04</v>
+      </c>
+      <c r="N25">
         <v>1000</v>
       </c>
-      <c r="N25">
-        <f t="shared" si="0"/>
-        <v>0.31666666666666654</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O25">
+        <f t="shared" si="0"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
         <v>52</v>
-      </c>
-      <c r="B26" t="s">
-        <v>53</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -1941,26 +1980,26 @@
       <c r="D26">
         <v>0.02</v>
       </c>
-      <c r="M26">
-        <v>0</v>
-      </c>
       <c r="N26">
-        <f t="shared" ref="N26:N28" si="1">C26-D26*20-E26*0.8-F26*0.6-H26*5+I26*15+J26/300</f>
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <f t="shared" si="0"/>
         <v>-0.4</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="N27">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C28">
         <v>-5</v>
@@ -1984,11 +2023,14 @@
         <v>-950</v>
       </c>
       <c r="M28">
+        <v>-0.25</v>
+      </c>
+      <c r="N28">
         <v>3000</v>
       </c>
-      <c r="N28">
-        <f t="shared" si="1"/>
-        <v>8.5833333333333357</v>
+      <c r="O28">
+        <f t="shared" si="0"/>
+        <v>8.7500000000000018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
because i forgot it's also a rework
- 9mm suppressors now in line with 5.56 suppressors in terms of effects
- mp5sd velocity fix (the suppressor still has no effect on velocity but now it subtracts a reasonable amount)
- +2 ergo for the naughty dog suppressors since they can't mount grips anymore
</commit_message>
<xml_diff>
--- a/changes/9mm-muzzles.xlsx
+++ b/changes/9mm-muzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F4441C-33C5-4041-AB30-EE0BB3E1314C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC9B5E7-A04B-4AF8-AE67-2BD3875E911D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1219,7 +1219,7 @@
         <v>0.06</v>
       </c>
       <c r="I5">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>30</v>
@@ -1229,7 +1229,7 @@
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
-        <v>-3.3000000000000007</v>
+        <v>-3.4500000000000006</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -1483,13 +1483,13 @@
         <v>-8</v>
       </c>
       <c r="H12">
-        <v>-0.05</v>
+        <v>-0.02</v>
       </c>
       <c r="I12">
         <v>0.06</v>
       </c>
       <c r="J12">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M12">
         <v>-0.05</v>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="O12">
         <f>C12-D12*20-E12*0.8-F12*0.6-H12*10+I12*15+J12/200-M12*5</f>
-        <v>7.5</v>
+        <v>7.0750000000000011</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1522,13 +1522,13 @@
         <v>-9</v>
       </c>
       <c r="H13">
-        <v>-0.1</v>
+        <v>-0.04</v>
       </c>
       <c r="I13">
         <v>0.12</v>
       </c>
       <c r="J13">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="M13">
         <v>-0.15</v>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="O13">
         <f>C13-D13*20-E13*0.8-F13*0.6-H13*10+I13*15+J13/200-M13*5</f>
-        <v>8.7999999999999972</v>
+        <v>7.9999999999999982</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
@@ -1549,7 +1549,7 @@
         <v>19</v>
       </c>
       <c r="C14">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="D14">
         <v>0.22</v>
@@ -1561,13 +1561,13 @@
         <v>-9</v>
       </c>
       <c r="H14">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="I14">
         <v>0.14000000000000001</v>
       </c>
       <c r="J14">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="M14">
         <v>-0.13</v>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="O14">
         <f t="shared" si="0"/>
-        <v>4.5999999999999996</v>
+        <v>5.5250000000000004</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
@@ -1588,7 +1588,7 @@
         <v>38</v>
       </c>
       <c r="C15">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="D15">
         <v>0.22</v>
@@ -1600,13 +1600,13 @@
         <v>-9</v>
       </c>
       <c r="H15">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="I15">
         <v>0.14000000000000001</v>
       </c>
       <c r="J15">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="M15">
         <v>-0.13</v>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="O15">
         <f t="shared" si="0"/>
-        <v>3.5999999999999996</v>
+        <v>4.5250000000000004</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1639,13 +1639,13 @@
         <v>-10</v>
       </c>
       <c r="H16">
-        <v>-0.2</v>
+        <v>-0.08</v>
       </c>
       <c r="I16">
         <v>0.13</v>
       </c>
       <c r="J16">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="M16">
         <v>-0.2</v>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="O16">
         <f t="shared" si="0"/>
-        <v>10.099999999999998</v>
+        <v>8.2749999999999986</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
@@ -1678,7 +1678,7 @@
         <v>-11</v>
       </c>
       <c r="H17">
-        <v>-0.12</v>
+        <v>-0.05</v>
       </c>
       <c r="I17">
         <v>0.14000000000000001</v>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="O17">
         <f t="shared" si="0"/>
-        <v>8.6999999999999993</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
@@ -1717,13 +1717,13 @@
         <v>-12</v>
       </c>
       <c r="H18">
-        <v>-0.15</v>
+        <v>-0.06</v>
       </c>
       <c r="I18">
         <v>0.15</v>
       </c>
       <c r="J18">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="M18">
         <v>-0.1</v>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="O18">
         <f t="shared" si="0"/>
-        <v>8.7999999999999989</v>
+        <v>7.5249999999999986</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
@@ -1756,13 +1756,13 @@
         <v>-12</v>
       </c>
       <c r="H19">
-        <v>-0.15</v>
+        <v>-0.06</v>
       </c>
       <c r="I19">
         <v>0.15</v>
       </c>
       <c r="J19">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="M19">
         <v>-0.1</v>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="O19">
         <f t="shared" si="0"/>
-        <v>8.7999999999999989</v>
+        <v>7.5249999999999986</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
@@ -1795,7 +1795,7 @@
         <v>-14</v>
       </c>
       <c r="H20">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="I20">
         <v>0.14000000000000001</v>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="O20">
         <f t="shared" si="0"/>
-        <v>4.8000000000000007</v>
+        <v>4.1000000000000014</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1883,12 +1883,6 @@
         <v>-0.6</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="O23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>47</v>
@@ -1909,13 +1903,13 @@
         <v>-8</v>
       </c>
       <c r="H24">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="I24">
         <v>0.09</v>
       </c>
       <c r="J24">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="M24">
         <v>-0.08</v>
@@ -1925,7 +1919,7 @@
       </c>
       <c r="O24">
         <f t="shared" si="0"/>
-        <v>9.1</v>
+        <v>8.4250000000000007</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
@@ -1948,13 +1942,13 @@
         <v>-2</v>
       </c>
       <c r="H25">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="I25">
         <v>0.05</v>
       </c>
       <c r="J25">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="M25">
         <v>-0.04</v>
@@ -1964,7 +1958,7 @@
       </c>
       <c r="O25">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.47499999999999992</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -1988,12 +1982,6 @@
         <v>-0.4</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="O27">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
@@ -2020,7 +2008,7 @@
         <v>0.15</v>
       </c>
       <c r="J28">
-        <v>-950</v>
+        <v>-180</v>
       </c>
       <c r="M28">
         <v>-0.25</v>
@@ -2030,7 +2018,7 @@
       </c>
       <c r="O28">
         <f t="shared" si="0"/>
-        <v>8.7500000000000018</v>
+        <v>12.600000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>